<commit_message>
some refactoring and clean up of old code
</commit_message>
<xml_diff>
--- a/ExcludeSymbolsList.xlsx
+++ b/ExcludeSymbolsList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\backup\code\stock_spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EF8FF7-5FF9-4154-9709-360046157069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CD9E25F-1D84-4748-8C69-C2DC1276AECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2220" windowWidth="22695" windowHeight="13980" xr2:uid="{F636D4DC-EADF-4245-B1CB-9C96FF26E68F}"/>
+    <workbookView xWindow="4995" yWindow="1155" windowWidth="21600" windowHeight="14055" xr2:uid="{F636D4DC-EADF-4245-B1CB-9C96FF26E68F}"/>
   </bookViews>
   <sheets>
     <sheet name="Exclusions" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="71">
   <si>
     <t>ExcludeSymbols</t>
   </si>
@@ -245,6 +245,9 @@
   </si>
   <si>
     <t>VIG</t>
+  </si>
+  <si>
+    <t>OC</t>
   </si>
 </sst>
 </file>
@@ -597,7 +600,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCCC010F-AF43-4C17-80F9-11DC7CE12A53}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -837,92 +840,97 @@
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>15</v>
+        <v>70</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>69</v>
+        <v>32</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>57</v>
+        <v>29</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>57</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>55</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A64">
-    <sortCondition ref="A2:A64"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A65">
+    <sortCondition ref="A2:A65"/>
   </sortState>
   <dataConsolidate/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>